<commit_message>
Refresh live data 2026-05-22T13:40Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -1,41 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17260" tabRatio="600" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Live Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cancel Curves" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CX Sales" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASD Sales" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Home Sales" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Producer Sales" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mepco Outstanding" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marketing Budget" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ops Staffing" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SG&amp;A" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financial Detail" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EBITDA Bridge" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financial Summary" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Covenants" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Credit View" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Log" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Economics" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality of Earnings" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Free Cash Flow" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Charts" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LBO Returns" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Process" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Live Data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Assumptions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sources" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Cancel Curves" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="CX Sales" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ASD Sales" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Home Sales" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Producer Sales" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Mepco Outstanding" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Marketing Budget" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Ops Staffing" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="SG&amp;A" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Debt" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Financial Detail" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="EBITDA Bridge" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Financial Summary" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Covenants" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Credit View" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="DCF" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Trading Comps" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Sensitivity" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Audit Log" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Unit Economics" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Quality of Earnings" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Free Cash Flow" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Charts" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Precedent Transactions" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="LBO Returns" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Process" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -591,13 +591,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -621,7 +621,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -645,7 +645,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -669,7 +669,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -693,7 +693,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -746,13 +746,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -775,14 +775,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -807,14 +807,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -839,14 +839,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -898,13 +898,13 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -927,14 +927,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -986,13 +986,13 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1016,7 +1016,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1040,7 +1040,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1093,7 +1093,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -1108,9 +1108,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1130,9 +1130,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1152,9 +1152,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1174,9 +1174,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-05-21T19:27:44Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-05-22T13:40:43Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-05-21T19:27:44Z</t>
+          <t>Last refreshed: 2026-05-22T13:40:43Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.67</v>
+        <v>4.57</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-05-21T19:27:44Z</t>
+          <t>2026-05-22T13:40:43Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-05-21T19:27:44Z</t>
+          <t>2026-05-22T13:40:43Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.53</v>
+        <v>0.49</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-05-21T19:27:44Z</t>
+          <t>2026-05-22T13:40:43Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-05-21T19:27:44Z</t>
+          <t>2026-05-22T13:40:43Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-05-21T19:27:44Z</t>
+          <t>2026-05-22T13:40:43Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-05-21T19:27:44Z</t>
+          <t>2026-05-22T13:40:43Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-05-21T19:27:44Z</t>
+          <t>2026-05-22T13:40:43Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-05-21T19:27:44Z</t>
+          <t>2026-05-22T13:40:43Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-05-21T19:27:44Z</t>
+          <t>2026-05-22T13:40:43Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-05-21T19:27:44Z</t>
+          <t>2026-05-22T13:40:43Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-05-21T19:27:44Z</t>
+          <t>2026-05-22T13:40:43Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>254.9400024414062</v>
+        <v>255.2799987792969</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.76499938964844</v>
+        <v>42.66999816894531</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>38.75</v>
+        <v>39.3849983215332</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>546.9849853515625</v>
+        <v>546.9149780273438</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>185.2615051269531</v>
+        <v>186.9499969482422</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-05-25T14:19Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-05-22T13:40:43Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-05-25T14:19:18Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-05-22T13:40:43Z</t>
+          <t>Last refreshed: 2026-05-25T14:19:18Z</t>
         </is>
       </c>
     </row>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-05-22T13:40:43Z</t>
+          <t>2026-05-25T14:19:18Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-05-22T13:40:43Z</t>
+          <t>2026-05-25T14:19:18Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.49</v>
+        <v>0.43</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-05-22T13:40:43Z</t>
+          <t>2026-05-25T14:19:18Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-05-22T13:40:43Z</t>
+          <t>2026-05-25T14:19:18Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-05-22T13:40:43Z</t>
+          <t>2026-05-25T14:19:18Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32547,7 +32547,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>53.3</v>
+        <v>49.8</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -32571,12 +32571,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-05-22T13:40:43Z</t>
+          <t>2026-05-25T14:19:18Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-05-22T13:40:43Z</t>
+          <t>2026-05-25T14:19:18Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-05-22T13:40:43Z</t>
+          <t>2026-05-25T14:19:18Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-05-22T13:40:43Z</t>
+          <t>2026-05-25T14:19:18Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-05-22T13:40:43Z</t>
+          <t>2026-05-25T14:19:18Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-05-22T13:40:43Z</t>
+          <t>2026-05-25T14:19:18Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>255.2799987792969</v>
+        <v>254.8200073242188</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.66999816894531</v>
+        <v>42.34999847412109</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>39.3849983215332</v>
+        <v>40.33000183105469</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>546.9149780273438</v>
+        <v>544.7999877929688</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>186.9499969482422</v>
+        <v>187.7899932861328</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-05-26T14:12Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-05-25T14:19:18Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-05-26T14:12:00Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-05-25T14:19:18Z</t>
+          <t>Last refreshed: 2026-05-26T14:12:00Z</t>
         </is>
       </c>
     </row>
@@ -32346,7 +32346,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-05-25T14:19:18Z</t>
+          <t>2026-05-26T14:12:00Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-05-25T14:19:18Z</t>
+          <t>2026-05-26T14:12:00Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32438,7 +32438,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-05-25T14:19:18Z</t>
+          <t>2026-05-26T14:12:00Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-05-25T14:19:18Z</t>
+          <t>2026-05-26T14:12:00Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-05-25T14:19:18Z</t>
+          <t>2026-05-26T14:12:00Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-05-25T14:19:18Z</t>
+          <t>2026-05-26T14:12:00Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-05-25T14:19:18Z</t>
+          <t>2026-05-26T14:12:00Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-05-25T14:19:18Z</t>
+          <t>2026-05-26T14:12:00Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-05-25T14:19:18Z</t>
+          <t>2026-05-26T14:12:00Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-05-25T14:19:18Z</t>
+          <t>2026-05-26T14:12:00Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-05-25T14:19:18Z</t>
+          <t>2026-05-26T14:12:00Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>254.8200073242188</v>
+        <v>256.2799987792969</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.34999847412109</v>
+        <v>43.04000091552734</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>40.33000183105469</v>
+        <v>41.84999847412109</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>544.7999877929688</v>
+        <v>551.760009765625</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>187.7899932861328</v>
+        <v>187.9781951904297</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-05-27T14:36Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-05-26T14:12:00Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-05-27T14:35:59Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-05-26T14:12:00Z</t>
+          <t>Last refreshed: 2026-05-27T14:35:59Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.57</v>
+        <v>4.56</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-05-26T14:12:00Z</t>
+          <t>2026-05-27T14:35:59Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-05-26T14:12:00Z</t>
+          <t>2026-05-27T14:35:59Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.43</v>
+        <v>0.49</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-05-26T14:12:00Z</t>
+          <t>2026-05-27T14:35:59Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-05-26T14:12:00Z</t>
+          <t>2026-05-27T14:35:59Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-05-26T14:12:00Z</t>
+          <t>2026-05-27T14:35:59Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-05-26T14:12:00Z</t>
+          <t>2026-05-27T14:35:59Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-05-26T14:12:00Z</t>
+          <t>2026-05-27T14:35:59Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-05-26T14:12:00Z</t>
+          <t>2026-05-27T14:35:59Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-05-26T14:12:00Z</t>
+          <t>2026-05-27T14:35:59Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-05-26T14:12:00Z</t>
+          <t>2026-05-27T14:35:59Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-05-26T14:12:00Z</t>
+          <t>2026-05-27T14:35:59Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>256.2799987792969</v>
+        <v>256.1749877929688</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>43.04000091552734</v>
+        <v>43.29499816894531</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>41.84999847412109</v>
+        <v>42.64500045776367</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>551.760009765625</v>
+        <v>559.5750122070312</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>187.9781951904297</v>
+        <v>191.4750061035156</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-05-28T14:50Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-05-27T14:35:59Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-05-28T14:50:52Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-05-27T14:35:59Z</t>
+          <t>Last refreshed: 2026-05-28T14:50:52Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.56</v>
+        <v>4.5</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-05-27T14:35:59Z</t>
+          <t>2026-05-28T14:50:52Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-05-27T14:35:59Z</t>
+          <t>2026-05-28T14:50:52Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.49</v>
+        <v>0.48</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-05-27T14:35:59Z</t>
+          <t>2026-05-28T14:50:52Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32455,7 +32455,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>16.696</v>
+        <v>16.318</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -32479,12 +32479,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-05-27T14:35:59Z</t>
+          <t>2026-05-28T14:50:52Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-05-27T14:35:59Z</t>
+          <t>2026-05-28T14:50:52Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-05-27T14:35:59Z</t>
+          <t>2026-05-28T14:50:52Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-05-27T14:35:59Z</t>
+          <t>2026-05-28T14:50:52Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-05-27T14:35:59Z</t>
+          <t>2026-05-28T14:50:52Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-05-27T14:35:59Z</t>
+          <t>2026-05-28T14:50:52Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-05-27T14:35:59Z</t>
+          <t>2026-05-28T14:50:52Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-05-27T14:35:59Z</t>
+          <t>2026-05-28T14:50:52Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>256.1749877929688</v>
+        <v>251.2599945068359</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>43.29499816894531</v>
+        <v>42.6150016784668</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>42.64500045776367</v>
+        <v>43.09000015258789</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>559.5750122070312</v>
+        <v>554.6099853515625</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>191.4750061035156</v>
+        <v>187.3300018310547</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-05-29T14:17Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-05-28T14:50:52Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-05-29T14:17:09Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-05-28T14:50:52Z</t>
+          <t>Last refreshed: 2026-05-29T14:17:09Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.5</v>
+        <v>4.48</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-05-28T14:50:52Z</t>
+          <t>2026-05-29T14:17:09Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32392,7 +32392,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-05-28T14:50:52Z</t>
+          <t>2026-05-29T14:17:09Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.48</v>
+        <v>0.46</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-05-28T14:50:52Z</t>
+          <t>2026-05-29T14:17:09Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-05-28T14:50:52Z</t>
+          <t>2026-05-29T14:17:09Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-05-28T14:50:52Z</t>
+          <t>2026-05-29T14:17:09Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-05-28T14:50:52Z</t>
+          <t>2026-05-29T14:17:09Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-05-28T14:50:52Z</t>
+          <t>2026-05-29T14:17:09Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.51</v>
+        <v>6.53</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-05-28T14:50:52Z</t>
+          <t>2026-05-29T14:17:09Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-05-28T14:50:52Z</t>
+          <t>2026-05-29T14:17:09Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-05-28T14:50:52Z</t>
+          <t>2026-05-29T14:17:09Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-05-28T14:50:52Z</t>
+          <t>2026-05-29T14:17:09Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>251.2599945068359</v>
+        <v>247.1699981689453</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.6150016784668</v>
+        <v>43.04999923706055</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>43.09000015258789</v>
+        <v>44.4099006652832</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>554.6099853515625</v>
+        <v>569.4149780273438</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>187.3300018310547</v>
+        <v>187.5950012207031</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>